<commit_message>
Consumers pole replacement won ($300K) — move from pipeline to backlog
Consumers 2026 Pole Replacements awarded at $300K (up from the $276.5K
listed). Moved from probability-weighted pipeline to booked backlog at
100% across the model, deck, and dashboard:
- Phase 2 Backlog & Pipeline tab + Coverage Chart schedule arrays updated
- Deck: backlog table adds the won job (total $697K -> $997K); pipeline
  table marks it WON -> backlog (pending ex-won $1,900K / $950K weighted);
  coverage callouts 49%/21%/$1,724K -> 52%/30%/$1,609K; market slide and
  accounting slide EPC-paired figures updated ($12.6M -> $9.1M remaining)
- Dashboard coverage chart data + cov.png re-rendered

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0145i7FWr3AQEo26DBw1x2c4
</commit_message>
<xml_diff>
--- a/model/CVR_Model_Phase2_Forecast.xlsx
+++ b/model/CVR_Model_Phase2_Forecast.xlsx
@@ -239,7 +239,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Coverage Chart'!A34</f>
+              <f>'Coverage Chart'!A35</f>
             </strRef>
           </tx>
           <spPr>
@@ -257,7 +257,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Coverage Chart'!$B$34:$S$34</f>
+              <f>'Coverage Chart'!$B$35:$S$35</f>
             </numRef>
           </val>
         </ser>
@@ -938,7 +938,7 @@
         </is>
       </c>
       <c r="B5" s="26">
-        <f>(SUM(B34:S34)+SUM(B40:S40))/SUM(B41:S41)</f>
+        <f>(SUM(B35:S35)+SUM(B40:S40))/SUM(B41:S41)</f>
         <v/>
       </c>
     </row>
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>SUM(B41:S41)-SUM(B34:S34)-SUM(B40:S40)</f>
+        <f>SUM(B41:S41)-SUM(B35:S35)-SUM(B40:S40)</f>
         <v/>
       </c>
     </row>
@@ -1676,155 +1676,167 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>burn: Consumers — 2026 Pole Replacements</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="C34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="D34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="E34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="F34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="G34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="H34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="I34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="J34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="K34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="L34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="M34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="N34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="O34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="P34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="Q34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="R34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+      <c r="S34">
+        <f>'Backlog &amp; Pipeline'!$E14/18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Booked backlog</t>
         </is>
       </c>
-      <c r="B34">
-        <f>SUM(B25:B33)</f>
-        <v/>
-      </c>
-      <c r="C34">
-        <f>SUM(C25:C33)</f>
-        <v/>
-      </c>
-      <c r="D34">
-        <f>SUM(D25:D33)</f>
-        <v/>
-      </c>
-      <c r="E34">
-        <f>SUM(E25:E33)</f>
-        <v/>
-      </c>
-      <c r="F34">
-        <f>SUM(F25:F33)</f>
-        <v/>
-      </c>
-      <c r="G34">
-        <f>SUM(G25:G33)</f>
-        <v/>
-      </c>
-      <c r="H34">
-        <f>SUM(H25:H33)</f>
-        <v/>
-      </c>
-      <c r="I34">
-        <f>SUM(I25:I33)</f>
-        <v/>
-      </c>
-      <c r="J34">
-        <f>SUM(J25:J33)</f>
-        <v/>
-      </c>
-      <c r="K34">
-        <f>SUM(K25:K33)</f>
-        <v/>
-      </c>
-      <c r="L34">
-        <f>SUM(L25:L33)</f>
-        <v/>
-      </c>
-      <c r="M34">
-        <f>SUM(M25:M33)</f>
-        <v/>
-      </c>
-      <c r="N34">
-        <f>SUM(N25:N33)</f>
-        <v/>
-      </c>
-      <c r="O34">
-        <f>SUM(O25:O33)</f>
-        <v/>
-      </c>
-      <c r="P34">
-        <f>SUM(P25:P33)</f>
-        <v/>
-      </c>
-      <c r="Q34">
-        <f>SUM(Q25:Q33)</f>
-        <v/>
-      </c>
-      <c r="R34">
-        <f>SUM(R25:R33)</f>
-        <v/>
-      </c>
-      <c r="S34">
-        <f>SUM(S25:S33)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>bid: Frontier Make Ready</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>0</v>
-      </c>
-      <c r="C35" t="n">
-        <v>0</v>
+      <c r="B35">
+        <f>SUM(B25:B34)</f>
+        <v/>
+      </c>
+      <c r="C35">
+        <f>SUM(C25:C34)</f>
+        <v/>
       </c>
       <c r="D35">
-        <f>'Backlog &amp; Pipeline'!$C18*'Backlog &amp; Pipeline'!$D18/6</f>
+        <f>SUM(D25:D34)</f>
         <v/>
       </c>
       <c r="E35">
-        <f>'Backlog &amp; Pipeline'!$C18*'Backlog &amp; Pipeline'!$D18/6</f>
+        <f>SUM(E25:E34)</f>
         <v/>
       </c>
       <c r="F35">
-        <f>'Backlog &amp; Pipeline'!$C18*'Backlog &amp; Pipeline'!$D18/6</f>
+        <f>SUM(F25:F34)</f>
         <v/>
       </c>
       <c r="G35">
-        <f>'Backlog &amp; Pipeline'!$C18*'Backlog &amp; Pipeline'!$D18/6</f>
+        <f>SUM(G25:G34)</f>
         <v/>
       </c>
       <c r="H35">
-        <f>'Backlog &amp; Pipeline'!$C18*'Backlog &amp; Pipeline'!$D18/6</f>
+        <f>SUM(H25:H34)</f>
         <v/>
       </c>
       <c r="I35">
-        <f>'Backlog &amp; Pipeline'!$C18*'Backlog &amp; Pipeline'!$D18/6</f>
-        <v/>
-      </c>
-      <c r="J35" t="n">
-        <v>0</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" t="n">
-        <v>0</v>
+        <f>SUM(I25:I34)</f>
+        <v/>
+      </c>
+      <c r="J35">
+        <f>SUM(J25:J34)</f>
+        <v/>
+      </c>
+      <c r="K35">
+        <f>SUM(K25:K34)</f>
+        <v/>
+      </c>
+      <c r="L35">
+        <f>SUM(L25:L34)</f>
+        <v/>
+      </c>
+      <c r="M35">
+        <f>SUM(M25:M34)</f>
+        <v/>
+      </c>
+      <c r="N35">
+        <f>SUM(N25:N34)</f>
+        <v/>
+      </c>
+      <c r="O35">
+        <f>SUM(O25:O34)</f>
+        <v/>
+      </c>
+      <c r="P35">
+        <f>SUM(P25:P34)</f>
+        <v/>
+      </c>
+      <c r="Q35">
+        <f>SUM(Q25:Q34)</f>
+        <v/>
+      </c>
+      <c r="R35">
+        <f>SUM(R25:R34)</f>
+        <v/>
+      </c>
+      <c r="S35">
+        <f>SUM(S25:S34)</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>bid: Jacksonburg–Gateway (EPC-paired $3</t>
+          <t>bid: Frontier Make Ready</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1833,59 +1845,53 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0</v>
+      <c r="D36">
+        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/6</f>
+        <v/>
+      </c>
+      <c r="E36">
+        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/6</f>
+        <v/>
       </c>
       <c r="F36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
+        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/6</f>
         <v/>
       </c>
       <c r="G36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
+        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/6</f>
         <v/>
       </c>
       <c r="H36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
+        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/6</f>
         <v/>
       </c>
       <c r="I36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="J36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="K36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="L36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="M36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="N36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="O36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="P36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
-      </c>
-      <c r="Q36">
-        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/12</f>
-        <v/>
+        <f>'Backlog &amp; Pipeline'!$C19*'Backlog &amp; Pipeline'!$D19/6</f>
+        <v/>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" t="n">
+        <v>0</v>
+      </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>0</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -1897,7 +1903,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>bid: Rosehill–Rockport (EPC-paired $5.5</t>
+          <t>bid: Jacksonburg–Gateway (EPC-paired $3</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1970,7 +1976,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>bid: Joint Use Audit</t>
+          <t>bid: Rosehill–Rockport (EPC-paired $5.5</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1985,66 +1991,65 @@
       <c r="E38" t="n">
         <v>0</v>
       </c>
-      <c r="F38" t="n">
-        <v>0</v>
+      <c r="F38">
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
+        <v/>
       </c>
       <c r="G38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="H38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="I38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="J38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="K38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="L38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="M38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="N38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="O38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="P38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
         <v/>
       </c>
       <c r="Q38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
-        <v/>
-      </c>
-      <c r="R38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
-        <v/>
-      </c>
-      <c r="S38">
-        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/18</f>
-        <v/>
+        <f>'Backlog &amp; Pipeline'!$C21*'Backlog &amp; Pipeline'!$D21/12</f>
+        <v/>
+      </c>
+      <c r="R38" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>bid: 2026 Pole Replacements (EPC-paired</t>
+          <t>bid: Joint Use Audit</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2059,59 +2064,60 @@
       <c r="E39" t="n">
         <v>0</v>
       </c>
-      <c r="F39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
-        <v/>
+      <c r="F39" t="n">
+        <v>0</v>
       </c>
       <c r="G39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="H39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="I39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="J39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="K39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="L39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="M39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="N39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="O39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="P39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
         <v/>
       </c>
       <c r="Q39">
-        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/12</f>
-        <v/>
-      </c>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" t="n">
-        <v>0</v>
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
+        <v/>
+      </c>
+      <c r="R39">
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
+        <v/>
+      </c>
+      <c r="S39">
+        <f>'Backlog &amp; Pipeline'!$C22*'Backlog &amp; Pipeline'!$D22/18</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -2121,75 +2127,75 @@
         </is>
       </c>
       <c r="B40">
-        <f>SUM(B35:B39)*$B$3</f>
+        <f>SUM(B36:B39)*$B$3</f>
         <v/>
       </c>
       <c r="C40">
-        <f>SUM(C35:C39)*$B$3</f>
+        <f>SUM(C36:C39)*$B$3</f>
         <v/>
       </c>
       <c r="D40">
-        <f>SUM(D35:D39)*$B$3</f>
+        <f>SUM(D36:D39)*$B$3</f>
         <v/>
       </c>
       <c r="E40">
-        <f>SUM(E35:E39)*$B$3</f>
+        <f>SUM(E36:E39)*$B$3</f>
         <v/>
       </c>
       <c r="F40">
-        <f>SUM(F35:F39)*$B$3</f>
+        <f>SUM(F36:F39)*$B$3</f>
         <v/>
       </c>
       <c r="G40">
-        <f>SUM(G35:G39)*$B$3</f>
+        <f>SUM(G36:G39)*$B$3</f>
         <v/>
       </c>
       <c r="H40">
-        <f>SUM(H35:H39)*$B$3</f>
+        <f>SUM(H36:H39)*$B$3</f>
         <v/>
       </c>
       <c r="I40">
-        <f>SUM(I35:I39)*$B$3</f>
+        <f>SUM(I36:I39)*$B$3</f>
         <v/>
       </c>
       <c r="J40">
-        <f>SUM(J35:J39)*$B$3</f>
+        <f>SUM(J36:J39)*$B$3</f>
         <v/>
       </c>
       <c r="K40">
-        <f>SUM(K35:K39)*$B$3</f>
+        <f>SUM(K36:K39)*$B$3</f>
         <v/>
       </c>
       <c r="L40">
-        <f>SUM(L35:L39)*$B$3</f>
+        <f>SUM(L36:L39)*$B$3</f>
         <v/>
       </c>
       <c r="M40">
-        <f>SUM(M35:M39)*$B$3</f>
+        <f>SUM(M36:M39)*$B$3</f>
         <v/>
       </c>
       <c r="N40">
-        <f>SUM(N35:N39)*$B$3</f>
+        <f>SUM(N36:N39)*$B$3</f>
         <v/>
       </c>
       <c r="O40">
-        <f>SUM(O35:O39)*$B$3</f>
+        <f>SUM(O36:O39)*$B$3</f>
         <v/>
       </c>
       <c r="P40">
-        <f>SUM(P35:P39)*$B$3</f>
+        <f>SUM(P36:P39)*$B$3</f>
         <v/>
       </c>
       <c r="Q40">
-        <f>SUM(Q35:Q39)*$B$3</f>
+        <f>SUM(Q36:Q39)*$B$3</f>
         <v/>
       </c>
       <c r="R40">
-        <f>SUM(R35:R39)*$B$3</f>
+        <f>SUM(R36:R39)*$B$3</f>
         <v/>
       </c>
       <c r="S40">
-        <f>SUM(S35:S39)*$B$3</f>
+        <f>SUM(S36:S39)*$B$3</f>
         <v/>
       </c>
     </row>
@@ -6200,95 +6206,100 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="3" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>(new)</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Consumers — 2026 Pole Replacements</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="19">
+        <f>C14-D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Dec-27</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>WON — award $300K; EPC-paired $3.45M</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Total backlog remaining</t>
         </is>
       </c>
-      <c r="E14" s="24">
-        <f>SUM(E5:E13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="E15" s="24">
+        <f>SUM(E5:E14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>PIPELINE — pending bids (CVR scope)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Bid</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>CVR value</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Win prob.</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>Expected</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F18" s="4" t="inlineStr">
         <is>
           <t>Expected award</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>Frontier Make Ready</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>Steuben County REMC</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n">
-        <v>100</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E18" s="19">
-        <f>C18*D18</f>
-        <v/>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Q3-26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>Jacksonburg–Gateway (EPC-paired $3.55M)</t>
+          <t>Frontier Make Ready</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Hoosier Energy</t>
+          <t>Steuben County REMC</t>
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>0.5</v>
@@ -6299,14 +6310,14 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>Q4-26</t>
+          <t>Q3-26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>Rosehill–Rockport (EPC-paired $5.59M)</t>
+          <t>Jacksonburg–Gateway (EPC-paired $3.55M)</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -6315,7 +6326,7 @@
         </is>
       </c>
       <c r="C20" s="19" t="n">
-        <v>290</v>
+        <v>160</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>0.5</v>
@@ -6333,16 +6344,16 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Joint Use Audit</t>
+          <t>Rosehill–Rockport (EPC-paired $5.59M)</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Lansing Board of Water &amp; Light</t>
+          <t>Hoosier Energy</t>
         </is>
       </c>
       <c r="C21" s="19" t="n">
-        <v>1350</v>
+        <v>290</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>0.5</v>
@@ -6360,19 +6371,19 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>2026 Pole Replacements (EPC-paired $3.45M)</t>
+          <t>Joint Use Audit</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Consumers Energy</t>
+          <t>Lansing Board of Water &amp; Light</t>
         </is>
       </c>
       <c r="C22" s="19" t="n">
-        <v>276</v>
+        <v>1350</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>0.67</v>
+        <v>0.5</v>
       </c>
       <c r="E22" s="19">
         <f>C22*D22</f>
@@ -6418,7 +6429,7 @@
         </is>
       </c>
       <c r="E24" s="24">
-        <f>SUM(E18:E23)</f>
+        <f>SUM(E19:E23)</f>
         <v/>
       </c>
     </row>
@@ -6447,7 +6458,7 @@
         </is>
       </c>
       <c r="B28" s="19">
-        <f>E14+E24</f>
+        <f>E15+E24</f>
         <v/>
       </c>
     </row>
@@ -6878,7 +6889,7 @@
         </is>
       </c>
       <c r="B7" s="19">
-        <f>'Backlog &amp; Pipeline'!E14</f>
+        <f>'Backlog &amp; Pipeline'!E15</f>
         <v/>
       </c>
       <c r="C7" s="19" t="n">

</xml_diff>

<commit_message>
Add EPC at-scale (material-margin) business model to model + deck
Model a future-state where CVR performs $150M/yr EPC and captures the
engineering scope plus material margin while HWC keeps equipment and labor
margin. New 'EPC At-Scale Model' tab (drivers, material + engineering P&L,
combined CVR economics, per-project illustration, sensitivity grid) in the
Phase 2 workbook; new deck slide with the value-split bar and headline
economics (~$18.8M managed revenue, ~$7.6M operating income, 6.3x the goal).
Drivers: 35% materials share, 13% material margin (net ~2 pts carry), 8%
engineering pull-through. Documented in PHASE2_FORECAST.md.
</commit_message>
<xml_diff>
--- a/model/CVR_Model_Phase2_Forecast.xlsx
+++ b/model/CVR_Model_Phase2_Forecast.xlsx
@@ -15,8 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash &amp; Note" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog &amp; Pipeline" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FY Summary" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Chart" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EPC At-Scale Model" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Chart" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,11 +26,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.0;(#,##0.0)"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00;($#,##0.00)"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot;×&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -106,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -135,6 +138,13 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -711,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="108" customWidth="1" min="1" max="1"/>
@@ -862,29 +872,43 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Checks             — anchors to the GL baseline and internal integrity checks.</t>
+          <t xml:space="preserve">  EPC At-Scale Model — revised business model: CVR earns engineering + material margin on a $150M/yr EPC program</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Coverage Chart     — native chart: forecast line vs backlog + pipeline areas, with a 1/0 toggle</t>
+          <t xml:space="preserve">                       (steady-state illustration; HWC keeps equipment + labor margin).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Checks             — anchors to the GL baseline and internal integrity checks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Coverage Chart     — native chart: forecast line vs backlog + pipeline areas, with a 1/0 toggle</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t xml:space="preserve">                       cell (B3) that includes or excludes the weighted pipeline live.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>COLOR KEY: blue = input · black = calculated · orange italics = assumption to confirm</t>
         </is>
@@ -896,6 +920,190 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="66" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Integrity checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>H1 revenue anchor ($K)</t>
+        </is>
+      </c>
+      <c r="B5" s="19">
+        <f>'FY Summary'!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="19" t="n">
+        <v>551</v>
+      </c>
+      <c r="D5" s="11">
+        <f>IF(ABS(B5-C5)&lt;=0.5,"TIES","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>H1 net income anchor ($K)</t>
+        </is>
+      </c>
+      <c r="B6" s="19">
+        <f>'FY Summary'!B9</f>
+        <v/>
+      </c>
+      <c r="C6" s="19" t="n">
+        <v>-320.5</v>
+      </c>
+      <c r="D6" s="11">
+        <f>IF(ABS(B6-C6)&lt;=0.5,"TIES","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Backlog remaining total ($K)</t>
+        </is>
+      </c>
+      <c r="B7" s="19">
+        <f>'Backlog &amp; Pipeline'!E15</f>
+        <v/>
+      </c>
+      <c r="C7" s="19" t="n">
+        <v>696.8</v>
+      </c>
+      <c r="D7" s="11">
+        <f>IF(ABS(B7-C7)&lt;=2.0,"TIES","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Note roll integrity: Dec-27 close = open − Σ op cash</t>
+        </is>
+      </c>
+      <c r="B8" s="19">
+        <f>'Cash &amp; Note'!S10</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>3436.6-SUM('Cash &amp; Note'!B9:S9)</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>IF(ABS(B8-C8)&lt;=0.1,"TIES","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Coverage ratio computed</t>
+        </is>
+      </c>
+      <c r="B9" s="19">
+        <f>'Backlog &amp; Pipeline'!B28</f>
+        <v/>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>&gt;0 expected</t>
+        </is>
+      </c>
+      <c r="D9" s="11">
+        <f>IF(B9&gt;0,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>MODEL LIMITS (read before presenting)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>• Revenue is capacity-driven; the coverage check disciplines it against booked work, but it is not a job-by-job burn schedule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• Direct-charge share (92%) mirrors the GL convention; when salary detail arrives, split wages properly by person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• The FTE path assumes hires are productive in month one — add ramp months per hire if that proves optimistic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Pipeline probabilities are placeholders at the 2026 win rate (67%) or 50% — Estimating should own these numbers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Escalation is off (card rate and wages flat through 2027) — turn on via the scalar inputs when the 2027 rate sheet lands.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -937,7 +1145,7 @@
           <t>Coverage of forecast</t>
         </is>
       </c>
-      <c r="B5" s="26">
+      <c r="B5" s="33">
         <f>(SUM(B35:S35)+SUM(B40:S40))/SUM(B41:S41)</f>
         <v/>
       </c>
@@ -948,7 +1156,7 @@
           <t>Gap to originate ($K)</t>
         </is>
       </c>
-      <c r="B6" s="27">
+      <c r="B6" s="34">
         <f>SUM(B41:S41)-SUM(B35:S35)-SUM(B40:S40)</f>
         <v/>
       </c>
@@ -6808,176 +7016,699 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="66" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Integrity checks</t>
+          <t>Revised Business Model — EPC at Scale: CVR earns engineering + material margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Steady-state illustration at $150M/yr EPC (NOT the near-term forecast). CVR takes engineering scope + material margin; HWC keeps equipment + labor margin. Blue = input; grey = calculated.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Expected</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DRIVERS — edit the blue cells</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>H1 revenue anchor ($K)</t>
-        </is>
-      </c>
-      <c r="B5" s="19">
-        <f>'FY Summary'!B5</f>
-        <v/>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>551</v>
-      </c>
-      <c r="D5" s="11">
-        <f>IF(ABS(B5-C5)&lt;=0.5,"TIES","CHECK")</f>
-        <v/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EPC program volume ($M/yr)</t>
+        </is>
+      </c>
+      <c r="B5" s="26" t="n">
+        <v>150</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Consolidated EPC run-rate (HWC + CVR)</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>H1 net income anchor ($K)</t>
-        </is>
-      </c>
-      <c r="B6" s="19">
-        <f>'FY Summary'!B9</f>
-        <v/>
-      </c>
-      <c r="C6" s="19" t="n">
-        <v>-320.5</v>
-      </c>
-      <c r="D6" s="11">
-        <f>IF(ABS(B6-C6)&lt;=0.5,"TIES","CHECK")</f>
-        <v/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CVR materials share of EPC</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Materials through CVR; major equipment stays with HWC</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Backlog remaining total ($K)</t>
-        </is>
-      </c>
-      <c r="B7" s="19">
-        <f>'Backlog &amp; Pipeline'!E15</f>
-        <v/>
-      </c>
-      <c r="C7" s="19" t="n">
-        <v>696.8</v>
-      </c>
-      <c r="D7" s="11">
-        <f>IF(ABS(B7-C7)&lt;=2.0,"TIES","CHECK")</f>
-        <v/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Material gross margin</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>CVR procurement markup on materials</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Note roll integrity: Dec-27 close = open − Σ op cash</t>
-        </is>
-      </c>
-      <c r="B8" s="19">
-        <f>'Cash &amp; Note'!S10</f>
-        <v/>
-      </c>
-      <c r="C8" s="19">
-        <f>3436.6-SUM('Cash &amp; Note'!B9:S9)</f>
-        <v/>
-      </c>
-      <c r="D8" s="11">
-        <f>IF(ABS(B8-C8)&lt;=0.1,"TIES","CHECK")</f>
-        <v/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Procurement + WC carry (pts of flow)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Purchasing staff + working-capital carry</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Coverage ratio computed</t>
-        </is>
-      </c>
-      <c r="B9" s="19">
-        <f>'Backlog &amp; Pipeline'!B28</f>
-        <v/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Engineering pull-through (% of EPC)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0.08</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>&gt;0 expected</t>
-        </is>
-      </c>
-      <c r="D9" s="11">
-        <f>IF(B9&gt;0,"OK","CHECK")</f>
-        <v/>
+          <t>CVR engineering scope at this scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Engineering gross margin</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Engineering revenue less direct labor</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>MODEL LIMITS (read before presenting)</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Engineering operating margin</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Engineering OI as % of eng revenue, at scale</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>• Revenue is capacity-driven; the coverage check disciplines it against booked work, but it is not a job-by-job burn schedule.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• Direct-charge share (92%) mirrors the GL convention; when salary detail arrives, split wages properly by person.</t>
+          <t>Working-capital carry (days of flow)</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Days from paying suppliers to reimbursement</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• The FTE path assumes hires are productive in month one — add ramp months per hire if that proves optimistic.</t>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>MATERIAL PROCUREMENT — CVR as principal ($M)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• Pipeline probabilities are placeholders at the 2026 win rate (67%) or 50% — Estimating should own these numbers.</t>
-        </is>
+          <t>Materials revenue (billed)</t>
+        </is>
+      </c>
+      <c r="B15" s="27">
+        <f>B5*B6</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• Escalation is off (card rate and wages flat through 2027) — turn on via the scalar inputs when the 2027 rate sheet lands.</t>
+          <t>Materials cost (COGS, at cost)</t>
+        </is>
+      </c>
+      <c r="B16" s="27">
+        <f>B15*(1-B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Material gross margin</t>
+        </is>
+      </c>
+      <c r="B17" s="27">
+        <f>B15*B7</f>
+        <v/>
+      </c>
+      <c r="C17" s="28">
+        <f>B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Procurement + working-capital cost</t>
+        </is>
+      </c>
+      <c r="B18" s="27">
+        <f>B15*B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Material net contribution</t>
+        </is>
+      </c>
+      <c r="B19" s="29">
+        <f>B17-B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ENGINEERING SERVICES ($M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Engineering revenue</t>
+        </is>
+      </c>
+      <c r="B22" s="27">
+        <f>B5*B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Engineering gross profit</t>
+        </is>
+      </c>
+      <c r="B23" s="27">
+        <f>B22*B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Engineering operating income</t>
+        </is>
+      </c>
+      <c r="B24" s="29">
+        <f>B22*B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Engineering OpEx (= GP − OI)</t>
+        </is>
+      </c>
+      <c r="B25" s="27">
+        <f>B23-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>COMBINED CVR — STEADY STATE ($M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>CVR revenue — gross / principal basis</t>
+        </is>
+      </c>
+      <c r="B28" s="27">
+        <f>B22+B15</f>
+        <v/>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>CVR takes title to materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>CVR revenue — managed-margin basis</t>
+        </is>
+      </c>
+      <c r="B29" s="29">
+        <f>B22+B17</f>
+        <v/>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>engineering + material margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CVR gross profit</t>
+        </is>
+      </c>
+      <c r="B30" s="27">
+        <f>B23+B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Total operating cost</t>
+        </is>
+      </c>
+      <c r="B31" s="27">
+        <f>B25+B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>CVR operating income (OILI)</t>
+        </is>
+      </c>
+      <c r="B32" s="30">
+        <f>B30-B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>OI margin — managed revenue</t>
+        </is>
+      </c>
+      <c r="B33" s="10">
+        <f>B32/B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>OI margin — gross revenue</t>
+        </is>
+      </c>
+      <c r="B34" s="10">
+        <f>B32/B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Working-capital requirement ($M)</t>
+        </is>
+      </c>
+      <c r="B35" s="27">
+        <f>B15*B12/365</f>
+        <v/>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>materials flow × carry days</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>CONTEXT vs TODAY &amp; THE YEAR-2 GOAL ($M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>CVR revenue today (managed, ~FY26)</t>
+        </is>
+      </c>
+      <c r="B38" s="26" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>current baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>This model — managed revenue</t>
+        </is>
+      </c>
+      <c r="B39" s="27">
+        <f>B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Year-2 goal operating profit ($6M × 20%)</t>
+        </is>
+      </c>
+      <c r="B40" s="26" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>This model — operating income</t>
+        </is>
+      </c>
+      <c r="B41" s="27">
+        <f>B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Multiple of the Year-2 goal profit</t>
+        </is>
+      </c>
+      <c r="B42" s="31">
+        <f>B32/B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>PER-PROJECT ILLUSTRATION — a $3.45M EPC job ($M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>EPC job value</t>
+        </is>
+      </c>
+      <c r="B45" s="26" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>Consumers-paired size</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Materials (share of job)</t>
+        </is>
+      </c>
+      <c r="B46" s="27">
+        <f>B45*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>CVR material margin</t>
+        </is>
+      </c>
+      <c r="B47" s="27">
+        <f>B46*B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>CVR engineering scope</t>
+        </is>
+      </c>
+      <c r="B48" s="27">
+        <f>B45*B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>CVR total take on the job</t>
+        </is>
+      </c>
+      <c r="B49" s="29">
+        <f>B47+B48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>CVR take as % of job value</t>
+        </is>
+      </c>
+      <c r="B50" s="10">
+        <f>B49/B45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>vs engineering-only today ($0.30M)</t>
+        </is>
+      </c>
+      <c r="B51" s="27">
+        <f>B49-0.3</f>
+        <v/>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>uplift from adding material margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>SENSITIVITY — CVR operating income ($M): materials share × material margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>share ↓  /  margin →</t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="C54" s="32" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D54" s="32" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E54" s="32" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="32" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B55" s="27">
+        <f>$B$5*$A55*(B$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="C55" s="27">
+        <f>$B$5*$A55*(C$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D55" s="27">
+        <f>$B$5*$A55*(D$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="E55" s="27">
+        <f>$B$5*$A55*(E$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="32" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B56" s="27">
+        <f>$B$5*$A56*(B$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="C56" s="27">
+        <f>$B$5*$A56*(C$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D56" s="27">
+        <f>$B$5*$A56*(D$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="E56" s="27">
+        <f>$B$5*$A56*(E$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="32" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B57" s="27">
+        <f>$B$5*$A57*(B$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="C57" s="27">
+        <f>$B$5*$A57*(C$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D57" s="30">
+        <f>$B$5*$A57*(D$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="E57" s="27">
+        <f>$B$5*$A57*(E$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="32" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B58" s="27">
+        <f>$B$5*$A58*(B$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="C58" s="27">
+        <f>$B$5*$A58*(C$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D58" s="27">
+        <f>$B$5*$A58*(D$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="E58" s="27">
+        <f>$B$5*$A58*(E$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="32" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="B59" s="27">
+        <f>$B$5*$A59*(B$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="C59" s="27">
+        <f>$B$5*$A59*(C$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D59" s="27">
+        <f>$B$5*$A59*(D$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+      <c r="E59" s="27">
+        <f>$B$5*$A59*(E$54-$B$8)+$B$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>• Steady-state at $150M/yr EPC — a future-state illustration, not the 18-month forecast. Reaching it depends on the EPC ramp (BD origination + HWC delivery capacity).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>• Materials shown on a PRINCIPAL basis (CVR takes title): CVR recognizes ~$52.5M materials revenue and ~$45.7M COGS. On a managed-margin (agent) basis, CVR 'revenue' is engineering + material margin ≈ $18.8M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>• CVR carries material procurement and price/obsolescence risk plus ~$6.5M of working capital; the 2-pt carry cost is a placeholder — confirm payment terms and a financing line with USC/HWC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>• HWC retains equipment procurement and the labor/construction margin, so CVR participates in EPC economics without taking construction-execution risk.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CEO/COO ask slide + FY-Summary at-scale block; lead priorities with BD hire
Deck now closes on the investment ask: a dedicated BD resource (~$300K/yr
all-in) to convert AEP and FirstEnergy (both warm), with warm-target cards,
payback tiles (one EPC win covers it; $7.6M at-scale upside), and a decision
line. Priorities #1 becomes 'Fund the BD resource — now.'

Workbook: FY Summary surfaces the at-scale model (managed revenue, operating
income, OILI margin, multiple of goal) beside the near-term scenarios.
</commit_message>
<xml_diff>
--- a/model/CVR_Model_Phase2_Forecast.xlsx
+++ b/model/CVR_Model_Phase2_Forecast.xlsx
@@ -26,13 +26,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0.0;(#,##0.0)"/>
-    <numFmt numFmtId="168" formatCode="$#,##0.00;($#,##0.00)"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
     <numFmt numFmtId="169" formatCode="0.0&quot;×&quot;"/>
+    <numFmt numFmtId="170" formatCode="$#,##0.00;($#,##0.00)"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -109,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,12 +139,14 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1145,7 +1148,7 @@
           <t>Coverage of forecast</t>
         </is>
       </c>
-      <c r="B5" s="33">
+      <c r="B5" s="35">
         <f>(SUM(B35:S35)+SUM(B40:S40))/SUM(B41:S41)</f>
         <v/>
       </c>
@@ -1156,7 +1159,7 @@
           <t>Gap to originate ($K)</t>
         </is>
       </c>
-      <c r="B6" s="34">
+      <c r="B6" s="36">
         <f>SUM(B41:S41)-SUM(B35:S35)-SUM(B40:S40)</f>
         <v/>
       </c>
@@ -6699,7 +6702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6999,7 +7002,65 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>AT-SCALE EPC MODEL (future state — see 'EPC At-Scale Model' tab), $M</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>CVR managed revenue</t>
+        </is>
+      </c>
+      <c r="B22" s="26">
+        <f>'EPC At-Scale Model'!B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>CVR operating income (OILI)</t>
+        </is>
+      </c>
+      <c r="B23" s="27">
+        <f>'EPC At-Scale Model'!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>OILI margin (managed)</t>
+        </is>
+      </c>
+      <c r="B24" s="10">
+        <f>'EPC At-Scale Model'!B33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>Multiple of the $6M / 20% goal profit</t>
+        </is>
+      </c>
+      <c r="B25" s="28">
+        <f>'EPC At-Scale Model'!B42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>At-scale figures are $M and reflect $150M/yr EPC with CVR taking engineering + material margin (HWC keeps equipment + labor). A future-state target, not the FY27 forecast above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>The gap between FY27 forecast revenue and the $6M goal is structural (billable capacity), not effort: closing it requires the hiring ramp AND winning EPC-paired engineering at scale — see the utilization × realization grid in the Phase 1 workbook for the per-FTE ceiling math.</t>
         </is>
@@ -7054,7 +7115,7 @@
           <t>EPC program volume ($M/yr)</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="29" t="n">
         <v>150</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -7181,7 +7242,7 @@
           <t>Materials revenue (billed)</t>
         </is>
       </c>
-      <c r="B15" s="27">
+      <c r="B15" s="30">
         <f>B5*B6</f>
         <v/>
       </c>
@@ -7192,7 +7253,7 @@
           <t>Materials cost (COGS, at cost)</t>
         </is>
       </c>
-      <c r="B16" s="27">
+      <c r="B16" s="30">
         <f>B15*(1-B7)</f>
         <v/>
       </c>
@@ -7203,11 +7264,11 @@
           <t>Material gross margin</t>
         </is>
       </c>
-      <c r="B17" s="27">
+      <c r="B17" s="30">
         <f>B15*B7</f>
         <v/>
       </c>
-      <c r="C17" s="28">
+      <c r="C17" s="31">
         <f>B7</f>
         <v/>
       </c>
@@ -7218,7 +7279,7 @@
           <t>Procurement + working-capital cost</t>
         </is>
       </c>
-      <c r="B18" s="27">
+      <c r="B18" s="30">
         <f>B15*B8</f>
         <v/>
       </c>
@@ -7229,7 +7290,7 @@
           <t>Material net contribution</t>
         </is>
       </c>
-      <c r="B19" s="29">
+      <c r="B19" s="32">
         <f>B17-B18</f>
         <v/>
       </c>
@@ -7247,7 +7308,7 @@
           <t>Engineering revenue</t>
         </is>
       </c>
-      <c r="B22" s="27">
+      <c r="B22" s="30">
         <f>B5*B9</f>
         <v/>
       </c>
@@ -7258,7 +7319,7 @@
           <t>Engineering gross profit</t>
         </is>
       </c>
-      <c r="B23" s="27">
+      <c r="B23" s="30">
         <f>B22*B10</f>
         <v/>
       </c>
@@ -7269,7 +7330,7 @@
           <t>Engineering operating income</t>
         </is>
       </c>
-      <c r="B24" s="29">
+      <c r="B24" s="32">
         <f>B22*B11</f>
         <v/>
       </c>
@@ -7280,7 +7341,7 @@
           <t>Engineering OpEx (= GP − OI)</t>
         </is>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="30">
         <f>B23-B24</f>
         <v/>
       </c>
@@ -7298,7 +7359,7 @@
           <t>CVR revenue — gross / principal basis</t>
         </is>
       </c>
-      <c r="B28" s="27">
+      <c r="B28" s="30">
         <f>B22+B15</f>
         <v/>
       </c>
@@ -7314,7 +7375,7 @@
           <t>CVR revenue — managed-margin basis</t>
         </is>
       </c>
-      <c r="B29" s="29">
+      <c r="B29" s="32">
         <f>B22+B17</f>
         <v/>
       </c>
@@ -7330,7 +7391,7 @@
           <t>CVR gross profit</t>
         </is>
       </c>
-      <c r="B30" s="27">
+      <c r="B30" s="30">
         <f>B23+B17</f>
         <v/>
       </c>
@@ -7341,7 +7402,7 @@
           <t>Total operating cost</t>
         </is>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="30">
         <f>B25+B18</f>
         <v/>
       </c>
@@ -7352,7 +7413,7 @@
           <t>CVR operating income (OILI)</t>
         </is>
       </c>
-      <c r="B32" s="30">
+      <c r="B32" s="33">
         <f>B30-B31</f>
         <v/>
       </c>
@@ -7385,7 +7446,7 @@
           <t>Working-capital requirement ($M)</t>
         </is>
       </c>
-      <c r="B35" s="27">
+      <c r="B35" s="30">
         <f>B15*B12/365</f>
         <v/>
       </c>
@@ -7408,7 +7469,7 @@
           <t>CVR revenue today (managed, ~FY26)</t>
         </is>
       </c>
-      <c r="B38" s="26" t="n">
+      <c r="B38" s="29" t="n">
         <v>1.42</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7423,7 +7484,7 @@
           <t>This model — managed revenue</t>
         </is>
       </c>
-      <c r="B39" s="27">
+      <c r="B39" s="30">
         <f>B29</f>
         <v/>
       </c>
@@ -7434,7 +7495,7 @@
           <t>Year-2 goal operating profit ($6M × 20%)</t>
         </is>
       </c>
-      <c r="B40" s="26" t="n">
+      <c r="B40" s="29" t="n">
         <v>1.2</v>
       </c>
     </row>
@@ -7444,7 +7505,7 @@
           <t>This model — operating income</t>
         </is>
       </c>
-      <c r="B41" s="27">
+      <c r="B41" s="30">
         <f>B32</f>
         <v/>
       </c>
@@ -7455,7 +7516,7 @@
           <t>Multiple of the Year-2 goal profit</t>
         </is>
       </c>
-      <c r="B42" s="31">
+      <c r="B42" s="28">
         <f>B32/B40</f>
         <v/>
       </c>
@@ -7473,7 +7534,7 @@
           <t>EPC job value</t>
         </is>
       </c>
-      <c r="B45" s="26" t="n">
+      <c r="B45" s="29" t="n">
         <v>3.45</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -7488,7 +7549,7 @@
           <t>Materials (share of job)</t>
         </is>
       </c>
-      <c r="B46" s="27">
+      <c r="B46" s="30">
         <f>B45*B6</f>
         <v/>
       </c>
@@ -7499,7 +7560,7 @@
           <t>CVR material margin</t>
         </is>
       </c>
-      <c r="B47" s="27">
+      <c r="B47" s="30">
         <f>B46*B7</f>
         <v/>
       </c>
@@ -7510,7 +7571,7 @@
           <t>CVR engineering scope</t>
         </is>
       </c>
-      <c r="B48" s="27">
+      <c r="B48" s="30">
         <f>B45*B9</f>
         <v/>
       </c>
@@ -7521,7 +7582,7 @@
           <t>CVR total take on the job</t>
         </is>
       </c>
-      <c r="B49" s="29">
+      <c r="B49" s="32">
         <f>B47+B48</f>
         <v/>
       </c>
@@ -7543,7 +7604,7 @@
           <t>vs engineering-only today ($0.30M)</t>
         </is>
       </c>
-      <c r="B51" s="27">
+      <c r="B51" s="30">
         <f>B49-0.3</f>
         <v/>
       </c>
@@ -7566,120 +7627,120 @@
           <t>share ↓  /  margin →</t>
         </is>
       </c>
-      <c r="B54" s="32" t="n">
+      <c r="B54" s="34" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="C54" s="32" t="n">
+      <c r="C54" s="34" t="n">
         <v>0.1</v>
       </c>
-      <c r="D54" s="32" t="n">
+      <c r="D54" s="34" t="n">
         <v>0.13</v>
       </c>
-      <c r="E54" s="32" t="n">
+      <c r="E54" s="34" t="n">
         <v>0.16</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="32" t="n">
+      <c r="A55" s="34" t="n">
         <v>0.25</v>
       </c>
-      <c r="B55" s="27">
+      <c r="B55" s="30">
         <f>$B$5*$A55*(B$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="C55" s="27">
+      <c r="C55" s="30">
         <f>$B$5*$A55*(C$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="D55" s="27">
+      <c r="D55" s="30">
         <f>$B$5*$A55*(D$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="E55" s="27">
+      <c r="E55" s="30">
         <f>$B$5*$A55*(E$54-$B$8)+$B$24</f>
         <v/>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="32" t="n">
+      <c r="A56" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="B56" s="27">
+      <c r="B56" s="30">
         <f>$B$5*$A56*(B$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="C56" s="27">
+      <c r="C56" s="30">
         <f>$B$5*$A56*(C$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="D56" s="27">
+      <c r="D56" s="30">
         <f>$B$5*$A56*(D$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="E56" s="27">
+      <c r="E56" s="30">
         <f>$B$5*$A56*(E$54-$B$8)+$B$24</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="32" t="n">
+      <c r="A57" s="34" t="n">
         <v>0.35</v>
       </c>
-      <c r="B57" s="27">
+      <c r="B57" s="30">
         <f>$B$5*$A57*(B$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="C57" s="27">
+      <c r="C57" s="30">
         <f>$B$5*$A57*(C$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="D57" s="30">
+      <c r="D57" s="33">
         <f>$B$5*$A57*(D$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="E57" s="27">
+      <c r="E57" s="30">
         <f>$B$5*$A57*(E$54-$B$8)+$B$24</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="32" t="n">
+      <c r="A58" s="34" t="n">
         <v>0.4</v>
       </c>
-      <c r="B58" s="27">
+      <c r="B58" s="30">
         <f>$B$5*$A58*(B$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="C58" s="27">
+      <c r="C58" s="30">
         <f>$B$5*$A58*(C$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="D58" s="27">
+      <c r="D58" s="30">
         <f>$B$5*$A58*(D$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="E58" s="27">
+      <c r="E58" s="30">
         <f>$B$5*$A58*(E$54-$B$8)+$B$24</f>
         <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="32" t="n">
+      <c r="A59" s="34" t="n">
         <v>0.45</v>
       </c>
-      <c r="B59" s="27">
+      <c r="B59" s="30">
         <f>$B$5*$A59*(B$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="C59" s="27">
+      <c r="C59" s="30">
         <f>$B$5*$A59*(C$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="D59" s="27">
+      <c r="D59" s="30">
         <f>$B$5*$A59*(D$54-$B$8)+$B$24</f>
         <v/>
       </c>
-      <c r="E59" s="27">
+      <c r="E59" s="30">
         <f>$B$5*$A59*(E$54-$B$8)+$B$24</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Update model, deck, and dashboard to the 7/25/2026 CVR/EPC KPI package
Reconcile to the week-ending 7/25 package: team billable utilization 59.0% ->
60.8% with refreshed per-person hours/billable %; Consumers pole award booked
at its official $276.45K CVR value (was $300K); win rate 67% -> 69%; backlog
total $997K -> $973K; Renaissance 345kV off hold and new MEC VanMeter 161kV
pursuit both now in bid (Sep-26, EPC-paired). Refresh KPI dates to 7/25 and
re-render utilization/coverage charts. H1 financials, BD hours, and MEC EPC
values are unchanged. Also make render_deck_charts merge the manifest so the
separately-rendered margin chart survives a re-render.
</commit_message>
<xml_diff>
--- a/model/CVR_Model_Phase2_Forecast.xlsx
+++ b/model/CVR_Model_Phase2_Forecast.xlsx
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="B9" s="19">
-        <f>'Backlog &amp; Pipeline'!B28</f>
+        <f>'Backlog &amp; Pipeline'!B29</f>
         <v/>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1090,7 +1090,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• Pipeline probabilities are placeholders at the 2026 win rate (67%) or 50% — Estimating should own these numbers.</t>
+          <t>• Pipeline probabilities are placeholders at the 2026 win rate (69%) or 50% — Estimating should own these numbers.</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6087,7 +6087,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Backlog = remaining PO value on active jobs (KPI scorecard 7/11/26). Pipeline = pending bids × win probability.</t>
+          <t>Backlog = remaining PO value on active jobs (KPI scorecard 7/25/26). Pipeline = pending bids × win probability.</t>
         </is>
       </c>
     </row>
@@ -6428,7 +6428,7 @@
         </is>
       </c>
       <c r="C14" s="19" t="n">
-        <v>300</v>
+        <v>276.45</v>
       </c>
       <c r="D14" s="19" t="n">
         <v>0</v>
@@ -6444,7 +6444,7 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>WON — award $300K; EPC-paired $3.45M</t>
+          <t>WON — award $276K; EPC-paired $3.45M</t>
         </is>
       </c>
     </row>
@@ -6609,7 +6609,7 @@
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Renaissance 345kV Substation (ON HOLD)</t>
+          <t>Renaissance 345kV Substation (6 MOD switches)</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
@@ -6629,63 +6629,90 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>Sep-26 — in bid</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>VanMeter 161kV Substation (EPC-paired)</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>MEC (MidAmerican)</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="19">
+        <f>C24*D24</f>
+        <v/>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Sep-26 — in bid</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Total probability-weighted pipeline</t>
         </is>
       </c>
-      <c r="E24" s="24">
-        <f>SUM(E19:E23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="E25" s="24">
+        <f>SUM(E19:E24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>COVERAGE CHECK</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Forecast revenue, Jul-26 – Dec-27</t>
-        </is>
-      </c>
-      <c r="B27" s="19">
-        <f>'Forecast P&amp;L'!T6+'Forecast P&amp;L'!U6</f>
-        <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>Booked + expected work (backlog + weighted pipeline)</t>
+          <t>Forecast revenue, Jul-26 – Dec-27</t>
         </is>
       </c>
       <c r="B28" s="19">
-        <f>E15+E24</f>
+        <f>'Forecast P&amp;L'!T6+'Forecast P&amp;L'!U6</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
         <is>
+          <t>Booked + expected work (backlog + weighted pipeline)</t>
+        </is>
+      </c>
+      <c r="B29" s="19">
+        <f>E15+E25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
           <t>Coverage ratio</t>
         </is>
       </c>
-      <c r="B29" s="10">
-        <f>B28/B27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="B30" s="10">
+        <f>B29/B28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>Coverage below 100% is normal at an 18-month horizon — the gap is work still to be won. But if coverage falls much below ~60%, the forecast is leaning on unidentified sales; treat the gap as the BD target: it quantifies how much new work Estimating must originate beyond the current bid list.</t>
         </is>

</xml_diff>